<commit_message>
simplified control files, improved weighted profile statistics across MSRs (script 2), more Excel-friendly time series output (script 4)
</commit_message>
<xml_diff>
--- a/3_attributor_combiner/control_file_attributor_combiner.xlsx
+++ b/3_attributor_combiner/control_file_attributor_combiner.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vub-my.sharepoint.com/personal/sebastian_sterl_vub_be/Documents/Documenten/VUB Work Files/MSR code repo/3_attributor_combiner/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vub-my.sharepoint.com/personal/sebastian_sterl_vub_be/Documents/Documenten/VUB Work Files/26001 MSR tutorial/3_attributor_combiner/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="11_18DF63992554B54D256DBF0CDD0837AADD87DA8D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D09D2D0C-C7AD-498A-A274-9B4E6A84C215}"/>
+  <xr:revisionPtr revIDLastSave="150" documentId="11_18DF63992554B54D256DBF0CDD0837AADD87DA8D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{93C0C439-85CA-497F-9EFB-5EE46C663C1F}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="paths" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="40">
   <si>
     <t>parameters</t>
   </si>
@@ -37,15 +37,6 @@
     <t>wind_hub_height</t>
   </si>
   <si>
-    <t>Unit: meters</t>
-  </si>
-  <si>
-    <t>elevation_threshold</t>
-  </si>
-  <si>
-    <t>Unit: m.a.s.l.</t>
-  </si>
-  <si>
     <t>hours_in_year</t>
   </si>
   <si>
@@ -61,24 +52,15 @@
     <t>wind_loss_adjustment</t>
   </si>
   <si>
-    <t>2% outage losses and 15% array and wake losses. Units: %</t>
-  </si>
-  <si>
     <t>solarpv_loss_adjustment</t>
   </si>
   <si>
-    <t>4% outage losses and 4% inverter and cable losses. Units: %</t>
-  </si>
-  <si>
     <t>configurations</t>
   </si>
   <si>
     <t>run_code_for_solar_pv</t>
   </si>
   <si>
-    <t xml:space="preserve">Options=[0-No, 1-Yes]. </t>
-  </si>
-  <si>
     <t>run_code_for_solar_csp</t>
   </si>
   <si>
@@ -103,12 +85,6 @@
     <t>region_names.csv</t>
   </si>
   <si>
-    <t>file_name_resource_raster</t>
-  </si>
-  <si>
-    <t>GHI_2026</t>
-  </si>
-  <si>
     <t>file_name_cost_assumptions</t>
   </si>
   <si>
@@ -121,19 +97,109 @@
     <t>input_folder_datasets</t>
   </si>
   <si>
-    <t>C:\Users\mastt\OneDrive - VITO\Documents\21_WP1\RawData\model_supply_regions\workflow\inputs\2022 MSR Toolset Inputs\</t>
-  </si>
-  <si>
     <t>Folder path where input datasets are located.</t>
   </si>
   <si>
     <t>output_folder</t>
   </si>
   <si>
-    <t>C:\Dev\model_supply_regions\Model-Supply-Regions-MSR-Toolset\outputs\</t>
+    <t>C:\Users\adm_sesterl\OneDrive - Vrije Universiteit Brussel\Documenten\VUB Work Files\26001 MSR tutorial\inputs</t>
+  </si>
+  <si>
+    <t>C:\Users\adm_sesterl\OneDrive - Vrije Universiteit Brussel\Documenten\VUB Work Files\26001 MSR tutorial\outputs</t>
   </si>
   <si>
     <t>Folder path where output files are located.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Units: %. Standard: consider 2% outage losses and 15% array and wake losses. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Units: %. Standard: consider 4% outage losses and 4% inverter and cable losses. </t>
+  </si>
+  <si>
+    <t>Options=[0-No, 1-Yes]. Select one at a time.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">number of hours in a year </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>(invariant)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">number of days in a year </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>(invariant)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Unit: meters. </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Only for correct column naming in eventual output. Does not change calculations.</t>
+    </r>
+  </si>
+  <si>
+    <t>ECU_wind_speed_100m</t>
+  </si>
+  <si>
+    <t>file_name_resource_raster_solarpv</t>
+  </si>
+  <si>
+    <t>file_name_resource_raster_wind</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Resource raster naming (.tif file) in </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">inputs </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>folder</t>
+    </r>
+  </si>
+  <si>
+    <t>ECU_GHI</t>
   </si>
 </sst>
 </file>
@@ -144,7 +210,7 @@
     <numFmt numFmtId="164" formatCode="#,##0.000"/>
     <numFmt numFmtId="165" formatCode="#,##0.0000000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -162,6 +228,38 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="5"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="2" tint="-0.249977111117893"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -193,7 +291,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -241,13 +339,47 @@
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -265,7 +397,7 @@
   <autoFilter ref="A1:C3" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="paths"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="value"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="value" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="comments"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -273,8 +405,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table4" displayName="Table4" ref="A1:C4" totalsRowShown="0">
-  <autoFilter ref="A1:C4" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table4" displayName="Table4" ref="A1:C5" totalsRowShown="0">
+  <autoFilter ref="A1:C5" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="datasets"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="value"/>
@@ -297,11 +429,11 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table6" displayName="Table6" ref="A1:C8" totalsRowShown="0">
-  <autoFilter ref="A1:C8" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table6" displayName="Table6" ref="A1:C7" totalsRowShown="0">
+  <autoFilter ref="A1:C7" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="parameters"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="value"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="value" dataDxfId="0"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="comments"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -596,17 +728,17 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="45.81640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.36328125" style="10" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="49.54296875" style="10" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="53" style="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
@@ -617,30 +749,35 @@
     </row>
     <row r="2" spans="1:3" s="1" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>26</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:3" s="1" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>35</v>
+        <v>25</v>
+      </c>
+      <c r="B3" s="19" t="s">
+        <v>27</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" s="1" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="10"/>
       <c r="B4" s="10"/>
       <c r="C4" s="10"/>
+    </row>
+    <row r="5" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="10"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -655,17 +792,17 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="25" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="49.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -676,26 +813,40 @@
     </row>
     <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" t="s">
-        <v>25</v>
+        <v>36</v>
+      </c>
+      <c r="B2" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B3" t="s">
-        <v>27</v>
+        <v>37</v>
+      </c>
+      <c r="B3" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B4" t="s">
-        <v>29</v>
+        <v>18</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -721,7 +872,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B1" s="14" t="s">
         <v>1</v>
@@ -732,57 +883,57 @@
     </row>
     <row r="2" spans="1:3" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B2" s="15">
+        <v>11</v>
+      </c>
+      <c r="B2" s="18">
         <v>1</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:3" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3" s="15">
+        <v>12</v>
+      </c>
+      <c r="B3" s="18">
         <v>0</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:3" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B4" s="15">
+        <v>13</v>
+      </c>
+      <c r="B4" s="18">
         <v>0</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:3" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="15">
+        <v>14</v>
+      </c>
+      <c r="B5" s="18">
         <v>0</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:3" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B6" s="15">
         <v>1</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -801,9 +952,9 @@
   <dimension ref="A1:P8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15" style="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.81640625" style="11" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.7265625" style="10" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.54296875" style="10" customWidth="1"/>
+    <col min="2" max="2" width="14.90625" style="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="80.6328125" style="10" customWidth="1"/>
     <col min="4" max="4" width="27.81640625" style="11" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="33.453125" style="10" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="25.1796875" style="11" bestFit="1" customWidth="1"/>
@@ -819,7 +970,7 @@
     <col min="16" max="16" width="22.54296875" style="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -843,15 +994,15 @@
       <c r="O1" s="3"/>
       <c r="P1" s="5"/>
     </row>
-    <row r="2" spans="1:16" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" s="1" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="7">
-        <v>100</v>
+        <v>6</v>
+      </c>
+      <c r="B2" s="21">
+        <v>50</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D2" s="7"/>
       <c r="E2" s="6"/>
@@ -867,15 +1018,15 @@
       <c r="O2" s="7"/>
       <c r="P2" s="9"/>
     </row>
-    <row r="3" spans="1:16" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="7">
-        <v>3000</v>
+        <v>8</v>
+      </c>
+      <c r="B3" s="21">
+        <v>83</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="6"/>
@@ -891,14 +1042,16 @@
       <c r="O3" s="7"/>
       <c r="P3" s="9"/>
     </row>
-    <row r="4" spans="1:16" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="7">
-        <v>8760</v>
-      </c>
-      <c r="C4" s="7"/>
+        <v>9</v>
+      </c>
+      <c r="B4" s="21">
+        <v>92</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>30</v>
+      </c>
       <c r="D4" s="7"/>
       <c r="E4" s="6"/>
       <c r="F4" s="7"/>
@@ -913,14 +1066,16 @@
       <c r="O4" s="7"/>
       <c r="P4" s="9"/>
     </row>
-    <row r="5" spans="1:16" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="7">
-        <v>365</v>
-      </c>
-      <c r="C5" s="7"/>
+        <v>3</v>
+      </c>
+      <c r="B5" s="21">
+        <v>100</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>34</v>
+      </c>
       <c r="D5" s="7"/>
       <c r="E5" s="6"/>
       <c r="F5" s="7"/>
@@ -935,15 +1090,15 @@
       <c r="O5" s="7"/>
       <c r="P5" s="9"/>
     </row>
-    <row r="6" spans="1:16" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="7">
-        <v>50</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>10</v>
+        <v>4</v>
+      </c>
+      <c r="B6" s="22">
+        <v>8760</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>32</v>
       </c>
       <c r="D6" s="7"/>
       <c r="E6" s="6"/>
@@ -959,15 +1114,15 @@
       <c r="O6" s="7"/>
       <c r="P6" s="9"/>
     </row>
-    <row r="7" spans="1:16" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="7">
-        <v>83</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>12</v>
+        <v>5</v>
+      </c>
+      <c r="B7" s="22">
+        <v>365</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>33</v>
       </c>
       <c r="D7" s="7"/>
       <c r="E7" s="6"/>
@@ -983,16 +1138,10 @@
       <c r="O7" s="7"/>
       <c r="P7" s="9"/>
     </row>
-    <row r="8" spans="1:16" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" s="7">
-        <v>92</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>14</v>
-      </c>
+    <row r="8" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="10"/>
+      <c r="B8" s="11"/>
+      <c r="C8" s="10"/>
       <c r="D8" s="7"/>
       <c r="E8" s="6"/>
       <c r="F8" s="7"/>

</xml_diff>